<commit_message>
Extend Devarim 5786 sheet through Simchat Torah with page numbers
Regenerate Devarim 5786.xlsx over the explicit range 2026-07-13 ->
2026-10-04 (the Monday before parshat Devarim through Simchat Torah)
so it includes the High Holiday season readings (Yom Kippur, Sukkot,
Shmini Atzeret, V'Zot HaBerachah) that the --book run cut off at
Ha'azinu. Generated with the 5786 Etz Hayim page numbers / haftarot.

Fix three parsha names in the 5786 CSV to match HebCal's spelling
(Ki Tetzei -> Ki Teitzei, Nitzavim-Va-yeilekh -> Nitzavim-Vayeilech,
Vezot ha-B'rakhah -> Vezot Haberakhah); the mismatches were silently
dropping page numbers for those rows.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Devarim 5786.xlsx
+++ b/Devarim 5786.xlsx
@@ -24,6 +24,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosh Hashana II" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tzom Gedaliah" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tzom Gedaliah (Mincha)" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yom Kippur" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yom Kippur (Mincha)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vezot Haberakhah" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sukkot I (on Shabbat)" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sukkot II" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sukkot Final Day (Hoshana Raba)" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shmini Atzeret (on Shabbat)" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Erev Simchat Torah" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simchat Torah" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -508,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.43" customWidth="1" min="1" max="1"/>
@@ -1958,6 +1967,412 @@
       <c r="B103" s="3" t="inlineStr"/>
       <c r="C103" s="3" t="inlineStr"/>
       <c r="D103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>Sep 24</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t>13 Tishrei</t>
+        </is>
+      </c>
+      <c r="C104" s="1" t="inlineStr">
+        <is>
+          <t>Vezot Haberakhah</t>
+        </is>
+      </c>
+      <c r="D104" s="1" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:1-7 (7)</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr"/>
+      <c r="D105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:8-12 (5)</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr"/>
+      <c r="D106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:13-17 (5)</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr"/>
+      <c r="D107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr"/>
+      <c r="B108" s="3" t="inlineStr"/>
+      <c r="C108" s="3" t="inlineStr"/>
+      <c r="D108" s="3" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Sep 28</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>17 Tishrei</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Sukkot Chol ha-Moed Day 1</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:17-19 (3)</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr"/>
+      <c r="D110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:20-22 (3)</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr"/>
+      <c r="D111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:23-25 (3)</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:17-22 (6)</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr"/>
+      <c r="D113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr"/>
+      <c r="B114" s="3" t="inlineStr"/>
+      <c r="C114" s="3" t="inlineStr"/>
+      <c r="D114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Sep 29</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>18 Tishrei</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Sukkot Chol ha-Moed Day 2</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:20-22 (3)</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr"/>
+      <c r="D116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:23-25 (3)</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr"/>
+      <c r="D117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:26-28 (3)</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr"/>
+      <c r="D118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:20-25 (6)</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr"/>
+      <c r="D119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr"/>
+      <c r="B120" s="3" t="inlineStr"/>
+      <c r="C120" s="3" t="inlineStr"/>
+      <c r="D120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>Sep 30</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>19 Tishrei</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Sukkot Chol ha-Moed Day 3</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:23-25 (3)</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr"/>
+      <c r="D122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:26-28 (3)</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr"/>
+      <c r="D123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:29-31 (3)</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr"/>
+      <c r="D124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:23-28 (6)</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr"/>
+      <c r="D125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr"/>
+      <c r="B126" s="3" t="inlineStr"/>
+      <c r="C126" s="3" t="inlineStr"/>
+      <c r="D126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Oct 01</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>20 Tishrei</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Sukkot Chol ha-Moed Day 4</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:26-28 (3)</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr"/>
+      <c r="D128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:29-31 (3)</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr"/>
+      <c r="D129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:32-34 (3)</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr"/>
+      <c r="D130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 29:26-31 (6)</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr"/>
+      <c r="D131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr"/>
+      <c r="B132" s="3" t="inlineStr"/>
+      <c r="C132" s="3" t="inlineStr"/>
+      <c r="D132" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2323,7 +2738,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 54:1-54:10 (10)</t>
+          <t>Isaiah 54:1-10</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -2365,7 +2780,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1112</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -2381,7 +2796,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1138</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -2835,7 +3250,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 60:1-60:22 (22)</t>
+          <t>Isaiah 60:1–9</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -2877,7 +3292,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1140</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -2893,7 +3308,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1161</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -3347,7 +3762,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 61:10-63:9 (23)</t>
+          <t>Isaiah 61:10-62:5</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -3389,7 +3804,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1165</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -3405,7 +3820,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1180</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -3863,7 +4278,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Hosea 14:2-14:10, 2:15-2:27 (22)</t>
+          <t>Hosea 14:2-10</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -3905,7 +4320,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1185</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -3921,7 +4336,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1234</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -5880,6 +6295,940 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Yom Kippur</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>September 21</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 10</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat September 20</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 39 verses (parsha=34)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 16:1-6 (6)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 16:7-11 (5)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 16:12-17 (6)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 16:18-24 (7)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A5", "V")</f>
+        <v/>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 16:25-30 (6)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=A6", "VI")</f>
+        <v/>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 16:31-34 (4)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Numbers 29:7-11 (5)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Isaiah 57:14-58:14 (22)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Yom Kippur (Mincha)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>September 21</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 10</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat September 20</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur (Mincha)", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 30 verses (parsha=21)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur (Mincha)&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 18:1-5 (5)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur (Mincha)&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 18:6-21 (16)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Yom Kippur (Mincha)&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 18:22-30 (9)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Jonah 1:1-4:11, 7:18-7:20 (51)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6239,7 +7588,3282 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 1:1-1:27 (27)</t>
+          <t>Isaiah 1:10-17</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Torah page 981</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page 1001</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vezot Haberakhah</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>September 24</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 13</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat September 23</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Vezot Haberakhah", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 0 verses (parsha=0)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Torah page 1202</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Sukkot I (on Shabbat)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>September 26</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 15</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat September 25</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 57 verses (parsha=52)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 22:26-33 (8)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 23:1-3 (3)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 23:4-8 (5)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 23:9-14 (6)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A5", "V")</f>
+        <v/>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 23:15-22 (8)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A6", "VI")</f>
+        <v/>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 23:23-32 (10)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=A7", "VII")</f>
+        <v/>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 23:33-44 (12)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot I (on Shabbat)&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Numbers 29:12-16 (5)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Zechariah 14:1-14:21 (21)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Sukkot II</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>September 27</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 16</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat September 26</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 57 verses (parsha=52)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 22:26-23:3 (11)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 23:4-14 (11)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Leviticus 23:15-22 (8)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Leviticus 23:23-32 (10)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=A5", "V")</f>
+        <v/>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Leviticus 23:33-44 (12)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot II&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Numbers 29:12-16 (5)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>I Kings 8:2-8:21 (20)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Sukkot Final Day (Hoshana Raba)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>October 2</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 21</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat October 1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot Final Day (Hoshana Raba)", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 15 verses (parsha=15)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot Final Day (Hoshana Raba)&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Numbers 29:26-28 (3)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot Final Day (Hoshana Raba)&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Numbers 29:29-31 (3)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot Final Day (Hoshana Raba)&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Numbers 29:32-34 (3)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Sukkot Final Day (Hoshana Raba)&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Numbers 29:29-34 (6)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr"/>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Shmini Atzeret (on Shabbat)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>October 3</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 22</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat October 2</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 54 verses (parsha=48)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 14:22-29 (8)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Deuteronomy 15:1-18 (18)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Deuteronomy 15:19-23 (5)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 16:1-3 (3)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A5", "V")</f>
+        <v/>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Deuteronomy 16:4-8 (5)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A6", "VI")</f>
+        <v/>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Deuteronomy 16:9-12 (4)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=A7", "VII")</f>
+        <v/>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 16:13-17 (5)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Shmini Atzeret (on Shabbat)&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Numbers 29:35-30:1 (6)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>I Kings 8:54-8:66 (13)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Erev Simchat Torah</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>October 3</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 22</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat October 2</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Erev Simchat Torah", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 17 verses (parsha=17)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Erev Simchat Torah&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:1-7 (7)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Erev Simchat Torah&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:8-12 (5)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Erev Simchat Torah&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:13-17 (5)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Etz Hayyim</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 1</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Torah page</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>P'ticha 2</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Haftarah page</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Hagbah</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>G'lilah</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Country</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Israel</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Prayer for Peace</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Anim Zmerot</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Adon Olam</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15.43" customWidth="1" min="1" max="1"/>
+    <col width="32.57" customWidth="1" min="2" max="2"/>
+    <col width="25.57" customWidth="1" min="3" max="3"/>
+    <col width="25.57" customWidth="1" min="4" max="4"/>
+    <col width="25.57" customWidth="1" min="5" max="5"/>
+    <col width="62.43" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr"/>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Simchat Torah</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr"/>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>October 4</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Tishrei 23</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rabbi Amanda Russell</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Service leaders</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kabbalat Shabbat October 3</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>P'sukei D'zimrah</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shacharit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Musaf</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>if(ISNUMBER(SEARCH("Richman",$A$2)), "RDR default", "RAR default")</f>
+        <v/>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Torah Service</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Gabbai</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sam (default)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Distribute honors</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Todd (default)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read announcements</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Jerilyn (default)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Board hosts</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Torah(s) Scroll</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Gunther</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;view=both&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah", "Virtual Tikkun")</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Full kriyah - 81 verses (parsha=75)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Aliyah</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hebrew Name(s)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A1", "I")</f>
+        <v/>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:1-7 (7)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A2", "II")</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:8-12 (5)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A3", "III")</f>
+        <v/>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:13-17 (5)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A4", "IV")</f>
+        <v/>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:18-21 (4)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A5", "V")</f>
+        <v/>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:22-26 (5)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A6", "VI")</f>
+        <v/>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Deuteronomy 33:27-34:12 (15)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=A7", "VII")</f>
+        <v/>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Genesis 1:1-2:3 (34)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11">
+        <f>hyperlink("https://myvirtualtikkun.com/?shul=cbssf&amp;scroll="&amp;$B$13&amp;"&amp;parsha=Simchat Torah&amp;aliyah=M", "Maf")</f>
+        <v/>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Numbers 29:35-30:1 (6)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Haf</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Joshua 1:1-1:18 (18)</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -6751,7 +11375,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 40:1-40:26 (26)</t>
+          <t xml:space="preserve">Isaiah 40:1-11 </t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -6793,7 +11417,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1005</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -6809,7 +11433,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1033</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -8513,7 +13137,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 49:14-51:3 (27)</t>
+          <t>Isaiah 50:10 - 51:3</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -8555,7 +13179,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1037</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -8571,7 +13195,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1059</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -9025,7 +13649,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 54:11-55:5 (12)</t>
+          <t>Isaiah 54:11-17</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -9067,7 +13691,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1061</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -9083,7 +13707,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1085</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -9537,7 +14161,7 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Isaiah 51:12-52:12 (24)</t>
+          <t>Isaiah 52:1 - 8</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr"/>
@@ -9579,7 +14203,7 @@
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Torah page</t>
+          <t>Torah page 1088</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -9595,7 +14219,7 @@
       <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Haftarah page</t>
+          <t>Haftarah page 1109</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>

</xml_diff>